<commit_message>
Modified the linear baseline script interface.
</commit_message>
<xml_diff>
--- a/assets/step1_linear/Step1_linear_experiment_tracker.xlsx
+++ b/assets/step1_linear/Step1_linear_experiment_tracker.xlsx
@@ -594,7 +594,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>AWR_PRESET=h200_8gpu_kl0；H200 1×8卡；KL=0
+          <t>H200 1×8卡；KL=1e-4
 f(r)=max(r,0)；w=f(r)/mean_group(f(r))；Δw=w−1
 全组f=0时Δw=0；v_target=v_old+Δw(u−v_old)，u=noise−x0
 每卡batch=6；rollout batches=24；梯度累积=24（含10时刻为240次backward）
@@ -611,13 +611,13 @@
       <c r="G2" s="3" t="inlineStr">
         <is>
           <t>v-prediction
-MSE(vθ,v_target)+0·MSE(vθ,v_ref)
+MSE(vθ,v_target)+1e-4·MSE(vθ,v_ref)
 无alpha、无外部t权重</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>P0（默认）</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -637,12 +637,12 @@
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>scripts/run_sd3_step1_linear.sh</t>
+          <t>scripts/run_sd3_h200_8gpu_step1_linear_kl1e-4.sh</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
         <is>
-          <t>sd35_pickscore_h200_8gpu_linear_kl0</t>
+          <t>sd35_pickscore_h200_8gpu_linear_kl1e-4</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>AWR_PRESET=4090_16gpu_kl1e-4；4090 2×8卡；KL=1e-4
+          <t>4090 2×8卡；KL=1e-4
 f(r)=max(r,0)；w=f(r)/mean_group(f(r))；Δw=w−1
 全组f=0时Δw=0；v_target=v_old+Δw(u−v_old)，u=noise−x0
 每卡batch=6；rollout batches=12；梯度累积=12（含10时刻为120次backward）
@@ -712,7 +712,7 @@
       </c>
       <c r="N3" s="6" t="inlineStr">
         <is>
-          <t>scripts/run_sd3_step1_linear.sh</t>
+          <t>scripts/run_sd3_4090_16gpu_step1_linear_kl1e-4.sh</t>
         </is>
       </c>
       <c r="O3" s="6" t="inlineStr">
@@ -776,11 +776,11 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>TASK=pickscore AWR_PRESET=h200_8gpu_kl0 PER_DEVICE_BATCH=6 AWR_VARIANCE_GATE=false bash scripts/run_sd3_step1_linear.sh</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="65" customHeight="1">
+          <t>TASK=pickscore PER_DEVICE_BATCH=6 AWR_VARIANCE_GATE=false bash scripts/run_sd3_h200_8gpu_step1_linear_kl1e-4.sh</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="92" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
           <t>01</t>
@@ -788,12 +788,14 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>对应AWR日志</t>
+          <t>对应AWR配置与历史日志</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>logs/public/flowawr/sd35_pickscore_h200_8gpu_flowawr_kl0-r1/
+          <t>对齐 scripts/flowawr_exps/run_sd3_h200_8gpu_flowawr_kl1e-4.sh；repo目前无H200/KL=1e-4结果日志。
+历史KL=0日志仅供参考，不作为本次严格仅改f的对照：
+logs/public/flowawr/sd35_pickscore_h200_8gpu_flowawr_kl0-r1/
 logs/public/flowawr/sd35_pickscore_h200_8gpu_flowawr_kl0-r2/</t>
         </is>
       </c>
@@ -811,7 +813,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>outputs/step1_linear/sd35_pickscore_h200_8gpu_linear_kl0/checkpoints/</t>
+          <t>outputs/step1_linear/sd35_pickscore_h200_8gpu_linear_kl1e-4/checkpoints/</t>
         </is>
       </c>
     </row>
@@ -828,7 +830,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>logs/step1_linear/sd35_pickscore_h200_8gpu_linear_kl0_&lt;时间戳&gt;/</t>
+          <t>logs/step1_linear/sd35_pickscore_h200_8gpu_linear_kl1e-4_&lt;时间戳&gt;/</t>
         </is>
       </c>
     </row>
@@ -879,12 +881,12 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>TASK=pickscore AWR_PRESET=4090_16gpu_kl1e-4 PER_DEVICE_BATCH=6 AWR_VARIANCE_GATE=false NNODES=2 NPROC_PER_NODE=8 NODE_RANK=0 MASTER_ADDR=&lt;节点0地址&gt; bash scripts/run_sd3_step1_linear.sh
-TASK=pickscore AWR_PRESET=4090_16gpu_kl1e-4 PER_DEVICE_BATCH=6 AWR_VARIANCE_GATE=false NNODES=2 NPROC_PER_NODE=8 NODE_RANK=1 MASTER_ADDR=&lt;节点0地址&gt; bash scripts/run_sd3_step1_linear.sh</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="65" customHeight="1">
+          <t>TASK=pickscore PER_DEVICE_BATCH=6 AWR_VARIANCE_GATE=false NNODES=2 NPROC_PER_NODE=8 NODE_RANK=0 MASTER_ADDR="节点0实际IP" bash scripts/run_sd3_4090_16gpu_step1_linear_kl1e-4.sh
+TASK=pickscore PER_DEVICE_BATCH=6 AWR_VARIANCE_GATE=false NNODES=2 NPROC_PER_NODE=8 NODE_RANK=1 MASTER_ADDR="节点0实际IP" bash scripts/run_sd3_4090_16gpu_step1_linear_kl1e-4.sh</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="72" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
           <t>02</t>
@@ -897,7 +899,8 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>logs/public/flowawr/sd35_pickscore_4090_16gpu_flowawr_kl1e-4-r1/
+          <t>对齐 scripts/flowawr_exps/run_sd3_4090_16gpu_flowawr_kl1e-4.sh；已有同KL日志（历史完整参数仍需核对）：
+logs/public/flowawr/sd35_pickscore_4090_16gpu_flowawr_kl1e-4-r1/
 logs/public/flowawr/sd35_pickscore_4090_16gpu_flowawr_kl1e-4-r2/</t>
         </is>
       </c>
@@ -999,7 +1002,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Run 01 / H2008 KL0</t>
+          <t>Run 01 / H2008 KL1e-4</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -1031,7 +1034,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>相对各自AWR的唯一训练算法修改：原为exp(r/sigma_R)</t>
+          <t>相对各自KL=1e-4 AWR启动配置，仅替换f：原为exp(r/sigma_R)；H200暂无同KL结果日志</t>
         </is>
       </c>
     </row>
@@ -1065,7 +1068,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1e-4</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -1163,7 +1166,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>group_count=48已由四份AWR日志核实</t>
+          <t>历史四份AWR日志group_count=48，其中H200为KL=0；本次规模对齐KL=1e-4脚本</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1276,7 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>四份AWR日志gradient_update_times=1</t>
+          <t>当前配置每轮1次更新；历史四份AWR日志亦为1，但H200历史为KL=0</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1452,7 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>四份AWR日志variance_gate=0</t>
+          <t>当前PickScore默认false；历史四份AWR日志为0，其中H200为KL=0</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1544,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="43" customHeight="1">
+    <row r="26" ht="84" customHeight="1">
       <c r="A26" s="3" t="inlineStr">
         <is>
           <t>历史一致性边界</t>
@@ -1549,17 +1552,17 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>未保存完整config/argv；不能逐项证明历史覆盖参数与代码版本</t>
+          <t>对齐repo的H200/KL=1e-4 AWR脚本；暂无同KL结果日志；H200/KL=0历史结果不能作为本次严格仅改f对照</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>同左</t>
+          <t>对齐repo的4090/KL=1e-4 AWR脚本；已有同KL日志，但未存完整config/argv，历史覆盖参数与代码版本仍需核对</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>对齐当前repo的AWR preset；历史额外覆盖需要同步</t>
+          <t>两项均KL=1e-4且使用独立启动脚本；仅与对应同KL AWR配置比较时才是只改f</t>
         </is>
       </c>
     </row>
@@ -1618,7 +1621,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="43" customHeight="1">
+    <row r="2" ht="72" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>sd35_pickscore_h200_8gpu_flowawr_kl0-r1</t>
@@ -1638,11 +1641,11 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>最新可见值，不代表实验最终值/预算</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="43" customHeight="1">
+          <t>历史H200/KL=0记录，不作为本次Run01 KL=1e-4的严格仅改f对照；最新可见值，不代表实验最终值/预算</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="72" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
           <t>sd35_pickscore_h200_8gpu_flowawr_kl0-r2</t>
@@ -1662,7 +1665,7 @@
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>日志从210开始，不能当作完整从零独立运行</t>
+          <t>历史H200/KL=0记录，不作为本次Run01 KL=1e-4的严格仅改f对照；日志从210开始，不能当作完整从零独立运行</t>
         </is>
       </c>
     </row>
@@ -1745,7 +1748,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="48" customHeight="1">
+    <row r="2" ht="60" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
           <t>状态</t>
@@ -1753,7 +1756,7 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>通过：本地真实8GPU训练，退出码0，70/70项验收通过</t>
+          <t>历史KL=0缩量验证通过：本地真实8GPU训练，退出码0，70/70项验收通过；未验证本次KL=1e-4</t>
         </is>
       </c>
     </row>
@@ -1877,7 +1880,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="48" customHeight="1">
+    <row r="13" ht="84" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
           <t>范围限制</t>
@@ -1885,7 +1888,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>这是本地缩量测试；未验证H200/4090完整batch。setup.py的torch2.6.0未在此次运行中使用。正式Run01/02仍待运行。</t>
+          <t>这是历史KL=0本地缩量测试，不代表本次KL=1e-4已通过训练验证；未验证H200/4090完整batch。setup.py的torch2.6.0未在此次运行中使用。正式Run01/02均KL=1e-4，仍待运行。</t>
         </is>
       </c>
     </row>

</xml_diff>